<commit_message>
chore(data): refresh riib spreadsheet sync
</commit_message>
<xml_diff>
--- a/Data Pegawai dan Dosen RIIB.xlsx
+++ b/Data Pegawai dan Dosen RIIB.xlsx
@@ -2,11 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIIB" sheetId="1" r:id="Rb7fc7b914d764414"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RIIB" sheetId="1" r:id="R1396e7df0f0b431b"/>
   </x:sheets>
-  <x:definedNames>
-    <x:definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RIIB'!$A$1:$J$41</x:definedName>
-  </x:definedNames>
 </x:workbook>
 </file>
 
@@ -951,7 +948,7 @@
       </x:c>
       <x:c r="J12" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Belum</x:t>
+          <x:t xml:space="preserve">Sudah</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -1997,7 +1994,7 @@
       </x:c>
       <x:c r="J33" s="2" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Belum</x:t>
+          <x:t xml:space="preserve">Sudah</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -2406,7 +2403,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f920763c454772"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R62bbe83cb6b540ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
chore(data): fill indikator column colors
</commit_message>
<xml_diff>
--- a/Data Pegawai dan Dosen RIIB.xlsx
+++ b/Data Pegawai dan Dosen RIIB.xlsx
@@ -27,7 +27,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -37,6 +37,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor rgb="FFC00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor rgb="FF00B050"/>
       </patternFill>
     </fill>
   </fills>
@@ -52,7 +70,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -66,6 +84,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -142,9 +163,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RIIB_Table" displayName="RIIB_Table" ref="A1:J41" headerRowCount="1">
-  <autoFilter ref="A1:J41"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RIIB_Table" displayName="RIIB_Table" ref="A1:K41" headerRowCount="1">
+  <autoFilter ref="A1:K41"/>
+  <tableColumns count="11">
     <tableColumn id="1" name="KODE DOSEN"/>
     <tableColumn id="2" name="NAMA DOSEN"/>
     <tableColumn id="3" name="NIP"/>
@@ -155,6 +176,7 @@
     <tableColumn id="8" name="JAFUNG"/>
     <tableColumn id="9" name="TANGGAL TMT"/>
     <tableColumn id="10" name="STATUS PUBLIKASI"/>
+    <tableColumn id="11" name="INDIKATOR"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showRowStripes="1"/>
 </table>
@@ -459,11 +481,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K2" s="5" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -514,11 +532,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -569,11 +583,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -624,11 +634,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -679,11 +685,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -734,11 +736,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -789,11 +787,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -844,11 +838,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -895,11 +885,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -950,11 +936,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1001,11 +983,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>Hijau</t>
-        </is>
-      </c>
+      <c r="K12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1056,11 +1034,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1111,11 +1085,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1166,11 +1136,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1217,11 +1183,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1272,11 +1234,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1323,11 +1281,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1378,11 +1332,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1433,11 +1383,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1488,11 +1434,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1543,11 +1485,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1598,11 +1536,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1653,11 +1587,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1708,11 +1638,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1763,11 +1689,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1818,11 +1740,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1869,11 +1787,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -1924,11 +1838,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1979,11 +1889,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2034,11 +1940,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2089,11 +1991,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2144,11 +2042,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Hijau</t>
-        </is>
-      </c>
+      <c r="K33" s="7" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2199,11 +2093,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2254,11 +2144,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2309,11 +2195,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2364,11 +2246,7 @@
           <t>Sudah</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2419,11 +2297,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2474,11 +2348,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>Merah</t>
-        </is>
-      </c>
+      <c r="K39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2529,11 +2399,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2578,11 +2444,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>Kuning</t>
-        </is>
-      </c>
+      <c r="K41" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>